<commit_message>
Hornear hoja Despiece y Longitudes: ld, ldh, ganchos, cortes de barra y estribos (ya no salen en blanco)
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/DISENO-VIGAS-VIGUETAS-FINAL-v2.xlsx
+++ b/Proyectos/Diseno-Estructural/DISENO-VIGAS-VIGUETAS-FINAL-v2.xlsx
@@ -8255,27 +8255,27 @@
       </c>
       <c r="D10" s="16">
         <f>($E$5*1*0.8)/(1.1*SQRT($C$5)*2.5)*C10</f>
-        <v/>
+        <v>219.356836</v>
       </c>
       <c r="E10" s="16">
         <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C10</f>
-        <v/>
+        <v>285.1638868</v>
       </c>
       <c r="F10" s="19">
         <f>MAX(0.24*$E$5/SQRT($C$5)*C10,8*C10,150)</f>
-        <v/>
+        <v>180.9693897</v>
       </c>
       <c r="G10" s="16">
         <f>12*C10</f>
-        <v/>
+        <v>114</v>
       </c>
       <c r="H10" s="16">
         <f>MAX(6*C10,75)</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="I10" s="16">
         <f>6*C10</f>
-        <v/>
+        <v>57</v>
       </c>
     </row>
     <row r="11">
@@ -8289,27 +8289,27 @@
       </c>
       <c r="D11" s="16">
         <f>($E$5*1*0.8)/(1.1*SQRT($C$5)*2.5)*C11</f>
-        <v/>
+        <v>293.2454544</v>
       </c>
       <c r="E11" s="16">
         <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C11</f>
-        <v/>
+        <v>381.2190907</v>
       </c>
       <c r="F11" s="19">
         <f>MAX(0.24*$E$5/SQRT($C$5)*C11,8*C11,150)</f>
-        <v/>
+        <v>241.9274999</v>
       </c>
       <c r="G11" s="16">
         <f>12*C11</f>
-        <v/>
+        <v>152.4</v>
       </c>
       <c r="H11" s="16">
         <f>MAX(6*C11,75)</f>
-        <v/>
+        <v>76.2</v>
       </c>
       <c r="I11" s="16">
         <f>6*C11</f>
-        <v/>
+        <v>76.2</v>
       </c>
     </row>
     <row r="12">
@@ -8323,27 +8323,27 @@
       </c>
       <c r="D12" s="16">
         <f>($E$5*1*0.8)/(1.1*SQRT($C$5)*2.5)*C12</f>
-        <v/>
+        <v>367.1340728</v>
       </c>
       <c r="E12" s="16">
         <f>($E$5*1.3*0.8)/(1.1*SQRT($C$5)*2.5)*C12</f>
-        <v/>
+        <v>477.2742947</v>
       </c>
       <c r="F12" s="19">
         <f>MAX(0.24*$E$5/SQRT($C$5)*C12,8*C12,150)</f>
-        <v/>
+        <v>302.8856101</v>
       </c>
       <c r="G12" s="16">
         <f>12*C12</f>
-        <v/>
+        <v>190.8</v>
       </c>
       <c r="H12" s="16">
         <f>MAX(6*C12,75)</f>
-        <v/>
+        <v>95.4</v>
       </c>
       <c r="I12" s="16">
         <f>6*C12</f>
-        <v/>
+        <v>95.4</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="33">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="E17" s="16">
         <f>F11</f>
-        <v/>
+        <v>241.9274999</v>
       </c>
       <c r="F17" s="21" t="inlineStr">
         <is>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="G17" s="19">
         <f>(D17/4*1000+E17)/1000</f>
-        <v/>
+        <v>1.5169275</v>
       </c>
     </row>
     <row r="18">
@@ -8443,7 +8443,7 @@
       </c>
       <c r="E18" s="16">
         <f>F12</f>
-        <v/>
+        <v>302.8856101</v>
       </c>
       <c r="F18" s="21" t="inlineStr">
         <is>
@@ -8452,7 +8452,7 @@
       </c>
       <c r="G18" s="19">
         <f>(D18*1000+2*E18)/1000</f>
-        <v/>
+        <v>5.70577122</v>
       </c>
     </row>
     <row r="19">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="E19" s="16">
         <f>F10</f>
-        <v/>
+        <v>180.9693897</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
@@ -8480,7 +8480,7 @@
       </c>
       <c r="G19" s="19">
         <f>(D19/4*1000+E19)/1000</f>
-        <v/>
+        <v>1.45596939</v>
       </c>
     </row>
     <row r="20" ht="27.95" customHeight="1" s="33">
@@ -8499,7 +8499,7 @@
       </c>
       <c r="E20" s="16">
         <f>F10</f>
-        <v/>
+        <v>180.9693897</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="G20" s="19">
         <f>(D20*1000+2*E20)/1000</f>
-        <v/>
+        <v>5.461938779</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1" s="33">
@@ -8577,19 +8577,19 @@
       </c>
       <c r="F24" s="16">
         <f>2*D24</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="G24" s="19">
         <f>MIN(E24/4,6*15.9,150)</f>
-        <v/>
+        <v>85.65</v>
       </c>
       <c r="H24" s="19">
         <f>E24/2</f>
-        <v/>
+        <v>171.3</v>
       </c>
       <c r="I24" s="16">
         <f>2*((C24-2*$G$5)+(D24-2*$G$5))+2*MAX(10*9.5,75)</f>
-        <v/>
+        <v>1270</v>
       </c>
     </row>
     <row r="25">
@@ -8609,19 +8609,19 @@
       </c>
       <c r="F25" s="16">
         <f>2*D25</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="G25" s="19">
         <f>MIN(E25/4,6*15.9,150)</f>
-        <v/>
+        <v>85.65</v>
       </c>
       <c r="H25" s="19">
         <f>E25/2</f>
-        <v/>
+        <v>171.3</v>
       </c>
       <c r="I25" s="16">
         <f>2*((C25-2*$G$5)+(D25-2*$G$5))+2*MAX(10*9.5,75)</f>
-        <v/>
+        <v>1370</v>
       </c>
     </row>
     <row r="26">
@@ -8641,19 +8641,19 @@
       </c>
       <c r="F26" s="16">
         <f>2*D26</f>
-        <v/>
+        <v>680</v>
       </c>
       <c r="G26" s="19">
         <f>MIN(E26/4,6*15.9,150)</f>
-        <v/>
+        <v>76</v>
       </c>
       <c r="H26" s="19">
         <f>E26/2</f>
-        <v/>
+        <v>152</v>
       </c>
       <c r="I26" s="16">
         <f>2*((C26-2*$G$5)+(D26-2*$G$5))+2*MAX(10*9.5,75)</f>
-        <v/>
+        <v>850</v>
       </c>
     </row>
     <row r="28" ht="27.95" customHeight="1" s="33">

</xml_diff>

<commit_message>
Hornear hojas heredadas (Irregularidades, Viguetas Entrepiso/Cubierta): 209 celdas que salian en blanco -> ahora con valores. Auditoria: 0 blancos, todos los grupos cumplen
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/DISENO-VIGAS-VIGUETAS-FINAL-v2.xlsx
+++ b/Proyectos/Diseno-Estructural/DISENO-VIGAS-VIGUETAS-FINAL-v2.xlsx
@@ -1397,20 +1397,20 @@
       </c>
       <c r="D18" s="7">
         <f>MAX(E68:E72,H68:H72)</f>
-        <v/>
+        <v>1.023571884</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
           <t>1.20 / 1.40</t>
         </is>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="7" t="str">
         <f>IF(D18&gt;1.4,"Extrema",IF(D18&gt;1.2,"Si","No"))</f>
-        <v/>
+        <v>No</v>
       </c>
       <c r="G18" s="8">
         <f>IF(D18&gt;1.4,0.8,IF(D18&gt;1.2,0.9,1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J18" s="32" t="inlineStr">
         <is>
@@ -1431,20 +1431,20 @@
       </c>
       <c r="D19" s="7">
         <f>MAX(C42/C40,C43/C41)</f>
-        <v/>
+        <v>0.1657285804</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
           <t>0.15</t>
         </is>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="7" t="str">
         <f>IF(AND(C42/C40&gt;0.15,C43/C41&gt;0.15),"Si","No")</f>
-        <v/>
+        <v>No</v>
       </c>
       <c r="G19" s="8">
         <f>IF(AND(C42/C40&gt;0.15,C43/C41&gt;0.15),0.9,1)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1460,19 +1460,19 @@
       </c>
       <c r="D20" s="7">
         <f>C45</f>
-        <v/>
+        <v>27.03</v>
       </c>
       <c r="E20" s="7">
         <f>0.5*C40*C41</f>
-        <v/>
-      </c>
-      <c r="F20" s="7">
+        <v>292.617</v>
+      </c>
+      <c r="F20" s="7" t="str">
         <f>IF(C45&gt;0.5*C40*C41,"Si","No")</f>
-        <v/>
+        <v>No</v>
       </c>
       <c r="G20" s="8">
         <f>IF(C45&gt;0.5*C40*C41,0.9,1)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="G23" s="9">
         <f>MIN(G18:G22)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="33">
@@ -1603,20 +1603,20 @@
       </c>
       <c r="D27" s="7">
         <f>MIN(G52:G55)</f>
-        <v/>
+        <v>1.064936106</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
           <t>0.70 / 0.60</t>
         </is>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="7" t="str">
         <f>IF(D27&lt;0.6,"Extrema",IF(D27&lt;0.7,"Si","No"))</f>
-        <v/>
+        <v>No</v>
       </c>
       <c r="G27" s="8">
         <f>IF(D27&lt;0.6,0.8,IF(D27&lt;0.7,0.9,1))</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" s="33">
@@ -1632,20 +1632,20 @@
       </c>
       <c r="D28" s="7">
         <f>MAX(H60:H63)</f>
-        <v/>
+        <v>1.323326017</v>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
           <t>1.50</t>
         </is>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="7" t="str">
         <f>IF(D28&gt;1.5,"Si","No")</f>
-        <v/>
+        <v>No</v>
       </c>
       <c r="G28" s="8">
         <f>IF(D28&gt;1.5,0.9,1)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="G32" s="9">
         <f>MIN(G27:G31)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1" s="33">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="C36" s="9">
         <f>IF(E35="Si",1,0.75)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="38" ht="31.5" customHeight="1" s="33">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C44" s="7">
         <f>C40*C41</f>
-        <v/>
+        <v>585.234</v>
       </c>
     </row>
     <row r="45">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C46" s="10">
         <f>C13*G32*G23*C36</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="47" ht="57.95" customHeight="1" s="33">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="D52" s="7">
         <f>SUM(C52:C56)</f>
-        <v/>
+        <v>15128.72</v>
       </c>
       <c r="E52" s="7" t="n">
         <v>0.022</v>
       </c>
       <c r="F52" s="7">
         <f>D52/E52</f>
-        <v/>
+        <v>687669.0909</v>
       </c>
       <c r="G52" s="7">
         <f>F52/F53</f>
-        <v/>
+        <v>1.410636191</v>
       </c>
     </row>
     <row r="53">
@@ -1961,18 +1961,18 @@
       </c>
       <c r="D53" s="7">
         <f>SUM(C53:C56)</f>
-        <v/>
+        <v>14137.17</v>
       </c>
       <c r="E53" s="7" t="n">
         <v>0.029</v>
       </c>
       <c r="F53" s="7">
         <f>D53/E53</f>
-        <v/>
+        <v>487488.6207</v>
       </c>
       <c r="G53" s="7">
         <f>F53/F54</f>
-        <v/>
+        <v>1.087083105</v>
       </c>
     </row>
     <row r="54">
@@ -1984,18 +1984,18 @@
       </c>
       <c r="D54" s="7">
         <f>SUM(C54:C56)</f>
-        <v/>
+        <v>11659.37</v>
       </c>
       <c r="E54" s="7" t="n">
         <v>0.026</v>
       </c>
       <c r="F54" s="7">
         <f>D54/E54</f>
-        <v/>
+        <v>448437.3077</v>
       </c>
       <c r="G54" s="7">
         <f>F54/F55</f>
-        <v/>
+        <v>1.064936106</v>
       </c>
     </row>
     <row r="55">
@@ -2007,18 +2007,18 @@
       </c>
       <c r="D55" s="7">
         <f>SUM(C55:C56)</f>
-        <v/>
+        <v>8000.77</v>
       </c>
       <c r="E55" s="7" t="n">
         <v>0.019</v>
       </c>
       <c r="F55" s="7">
         <f>D55/E55</f>
-        <v/>
+        <v>421093.1579</v>
       </c>
       <c r="G55" s="7">
         <f>F55/F56</f>
-        <v/>
+        <v>1.870865889</v>
       </c>
     </row>
     <row r="56">
@@ -2030,14 +2030,14 @@
       </c>
       <c r="D56" s="7">
         <f>SUM(C56:C56)</f>
-        <v/>
+        <v>3151.11</v>
       </c>
       <c r="E56" s="7" t="n">
         <v>0.014</v>
       </c>
       <c r="F56" s="7">
         <f>D56/E56</f>
-        <v/>
+        <v>225079.2857</v>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
@@ -2093,11 +2093,11 @@
       </c>
       <c r="E60" s="7">
         <f>C60/C61</f>
-        <v/>
+        <v>0.7556716842</v>
       </c>
       <c r="H60" s="7">
         <f>E60</f>
-        <v/>
+        <v>0.7556716842</v>
       </c>
     </row>
     <row r="61">
@@ -2109,15 +2109,15 @@
       </c>
       <c r="D61" s="7">
         <f>C61/C60</f>
-        <v/>
+        <v>1.323326017</v>
       </c>
       <c r="E61" s="7">
         <f>C61/C62</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H61" s="7">
         <f>MAX(D61,E61)</f>
-        <v/>
+        <v>1.323326017</v>
       </c>
     </row>
     <row r="62">
@@ -2129,15 +2129,15 @@
       </c>
       <c r="D62" s="7">
         <f>C62/C61</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="E62" s="7">
         <f>C62/C63</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H62" s="7">
         <f>MAX(D62,E62)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D63" s="7">
         <f>C63/C62</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H63" s="7">
         <f>D63</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E68" s="7">
         <f>C68/((C68+D68)/2)</f>
-        <v/>
+        <v>1.023571884</v>
       </c>
       <c r="F68" s="7" t="n">
         <v>0.02097</v>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="H68" s="7">
         <f>F68/((F68+G68)/2)</f>
-        <v/>
+        <v>1.013288234</v>
       </c>
     </row>
     <row r="69">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="E69" s="7">
         <f>C69/((C69+D69)/2)</f>
-        <v/>
+        <v>1.022820801</v>
       </c>
       <c r="F69" s="7" t="n">
         <v>0.04338</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="H69" s="7">
         <f>F69/((F69+G69)/2)</f>
-        <v/>
+        <v>1.014143776</v>
       </c>
     </row>
     <row r="70">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E70" s="7">
         <f>C70/((C70+D70)/2)</f>
-        <v/>
+        <v>1.022321985</v>
       </c>
       <c r="F70" s="7" t="n">
         <v>0.0625</v>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="H70" s="7">
         <f>F70/((F70+G70)/2)</f>
-        <v/>
+        <v>1.014363386</v>
       </c>
     </row>
     <row r="71">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="E71" s="7">
         <f>C71/((C71+D71)/2)</f>
-        <v/>
+        <v>1.022007838</v>
       </c>
       <c r="F71" s="7" t="n">
         <v>0.07592</v>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="H71" s="7">
         <f>F71/((F71+G71)/2)</f>
-        <v/>
+        <v>1.014498564</v>
       </c>
     </row>
     <row r="72">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="E72" s="7">
         <f>C72/((C72+D72)/2)</f>
-        <v/>
+        <v>1.021769631</v>
       </c>
       <c r="F72" s="7" t="n">
         <v>0.08278000000000001</v>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H72" s="7">
         <f>F72/((F72+G72)/2)</f>
-        <v/>
+        <v>1.014522949</v>
       </c>
     </row>
   </sheetData>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="C16" s="19">
         <f>C8*1000-C11*1000-C12/2</f>
-        <v/>
+        <v>303.65</v>
       </c>
     </row>
     <row r="17">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="C17" s="19">
         <f>(1.2*C14+1.6*C15)*C10</f>
-        <v/>
+        <v>9.0624</v>
       </c>
     </row>
     <row r="18">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="C18" s="21">
         <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*C7*1000*C16</f>
-        <v/>
+        <v>151.825</v>
       </c>
     </row>
     <row r="19">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="C19" s="21">
         <f>0.17*SQRT(C5)*C7*1000*C16/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
     </row>
     <row r="20">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="C20" s="21">
         <f>0.75*1.1*C19</f>
-        <v/>
+        <v>33.80231387</v>
       </c>
     </row>
     <row r="22">
@@ -6185,19 +6185,19 @@
       </c>
       <c r="C25" s="19">
         <f>MIN(C24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>462.5</v>
       </c>
       <c r="D25" s="19">
         <f>MIN(D24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E25" s="19">
         <f>MIN(E24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="F25" s="19">
         <f>MIN(F24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
     </row>
     <row r="26">
@@ -6208,19 +6208,19 @@
       </c>
       <c r="C26" s="19">
         <f>$C$17*C24^2/10</f>
-        <v/>
+        <v>3.1016064</v>
       </c>
       <c r="D26" s="19">
         <f>$C$17*D24^2/10</f>
-        <v/>
+        <v>9.57216</v>
       </c>
       <c r="E26" s="19">
         <f>$C$17*E24^2/10</f>
-        <v/>
+        <v>17.9458176</v>
       </c>
       <c r="F26" s="19">
         <f>$C$17*F24^2/10</f>
-        <v/>
+        <v>20.8797696</v>
       </c>
     </row>
     <row r="27">
@@ -6231,19 +6231,19 @@
       </c>
       <c r="C27" s="19">
         <f>$C$17*C24^2/14</f>
-        <v/>
+        <v>2.215433143</v>
       </c>
       <c r="D27" s="19">
         <f>$C$17*D24^2/14</f>
-        <v/>
+        <v>6.837257143</v>
       </c>
       <c r="E27" s="19">
         <f>$C$17*E24^2/14</f>
-        <v/>
+        <v>12.81844114</v>
       </c>
       <c r="F27" s="19">
         <f>$C$17*F24^2/14</f>
-        <v/>
+        <v>14.91412114</v>
       </c>
     </row>
     <row r="28">
@@ -6254,19 +6254,19 @@
       </c>
       <c r="C28" s="19">
         <f>1.15*$C$17*C24/2</f>
-        <v/>
+        <v>9.640128</v>
       </c>
       <c r="D28" s="19">
         <f>1.15*$C$17*D24/2</f>
-        <v/>
+        <v>16.93536</v>
       </c>
       <c r="E28" s="19">
         <f>1.15*$C$17*E24/2</f>
-        <v/>
+        <v>23.188416</v>
       </c>
       <c r="F28" s="19">
         <f>1.15*$C$17*F24/2</f>
-        <v/>
+        <v>25.012224</v>
       </c>
     </row>
     <row r="29">
@@ -6288,19 +6288,19 @@
       </c>
       <c r="C30" s="16">
         <f>C27*1000000/(0.9*C25*$C$16^2)</f>
-        <v/>
+        <v>0.05772418781</v>
       </c>
       <c r="D30" s="16">
         <f>D27*1000000/(0.9*D25*$C$16^2)</f>
-        <v/>
+        <v>0.1029918469</v>
       </c>
       <c r="E30" s="16">
         <f>E27*1000000/(0.9*E25*$C$16^2)</f>
-        <v/>
+        <v>0.1930883833</v>
       </c>
       <c r="F30" s="16">
         <f>F27*1000000/(0.9*F25*$C$16^2)</f>
-        <v/>
+        <v>0.2246562985</v>
       </c>
     </row>
     <row r="31">
@@ -6311,19 +6311,19 @@
       </c>
       <c r="C31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*C30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0001376056186</v>
       </c>
       <c r="D31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*D30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0002457515699</v>
       </c>
       <c r="E31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*E30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0004616144332</v>
       </c>
       <c r="F31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*F30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0005374445961</v>
       </c>
     </row>
     <row r="32">
@@ -6334,19 +6334,19 @@
       </c>
       <c r="C32" s="16">
         <f>C31*C25*$C$16</f>
-        <v/>
+        <v>19.32507507</v>
       </c>
       <c r="D32" s="16">
         <f>D31*D25*$C$16</f>
-        <v/>
+        <v>59.69797136</v>
       </c>
       <c r="E32" s="16">
         <f>E31*E25*$C$16</f>
-        <v/>
+        <v>112.1353781</v>
       </c>
       <c r="F32" s="16">
         <f>F31*F25*$C$16</f>
-        <v/>
+        <v>130.5560413</v>
       </c>
     </row>
     <row r="33">
@@ -6357,19 +6357,19 @@
       </c>
       <c r="C33" s="16">
         <f>C32*$C$6/(0.85*$C$5*C25)</f>
-        <v/>
+        <v>0.7373637547</v>
       </c>
       <c r="D33" s="16">
         <f>D32*$C$6/(0.85*$C$5*D25)</f>
-        <v/>
+        <v>1.316867015</v>
       </c>
       <c r="E33" s="16">
         <f>E32*$C$6/(0.85*$C$5*E25)</f>
-        <v/>
+        <v>2.473574517</v>
       </c>
       <c r="F33" s="16">
         <f>F32*$C$6/(0.85*$C$5*F25)</f>
-        <v/>
+        <v>2.879912676</v>
       </c>
     </row>
     <row r="34">
@@ -6378,21 +6378,21 @@
           <t>a &lt;= hf ? (viga T)</t>
         </is>
       </c>
-      <c r="C34" s="18">
+      <c r="C34" s="18" t="str">
         <f>IF(C33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="D34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="D34" s="18" t="str">
         <f>IF(D33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="E34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="E34" s="18" t="str">
         <f>IF(E33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="F34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="F34" s="18" t="str">
         <f>IF(F33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
     </row>
     <row r="35">
@@ -6403,19 +6403,19 @@
       </c>
       <c r="C35" s="19">
         <f>MAX(C32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="D35" s="19">
         <f>MAX(D32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="E35" s="19">
         <f>MAX(E32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="F35" s="19">
         <f>MAX(F32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
     </row>
     <row r="36">
@@ -6426,19 +6426,19 @@
       </c>
       <c r="C36" s="19">
         <f>ROUNDUP(C35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D36" s="19">
         <f>ROUNDUP(D35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E36" s="19">
         <f>ROUNDUP(E35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F36" s="19">
         <f>ROUNDUP(F35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -6460,19 +6460,19 @@
       </c>
       <c r="C38" s="16">
         <f>C26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>0.2491760774</v>
       </c>
       <c r="D38" s="16">
         <f>D26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>0.7690057903</v>
       </c>
       <c r="E38" s="16">
         <f>E26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>1.441726595</v>
       </c>
       <c r="F38" s="16">
         <f>F26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>1.677433696</v>
       </c>
     </row>
     <row r="39">
@@ -6483,19 +6483,19 @@
       </c>
       <c r="C39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*C38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0005964149999</v>
       </c>
       <c r="D39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*D38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.001861542708</v>
       </c>
       <c r="E39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*E38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.003543472336</v>
       </c>
       <c r="F39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*F38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.00414552547</v>
       </c>
     </row>
     <row r="40">
@@ -6506,19 +6506,19 @@
       </c>
       <c r="C40" s="16">
         <f>C39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>27.16521221</v>
       </c>
       <c r="D40" s="16">
         <f>D39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>84.78861649</v>
       </c>
       <c r="E40" s="16">
         <f>E39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>161.3963062</v>
       </c>
       <c r="F40" s="16">
         <f>F39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>188.8183213</v>
       </c>
     </row>
     <row r="41">
@@ -6529,19 +6529,19 @@
       </c>
       <c r="C41" s="19">
         <f>MAX(C40,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="D41" s="19">
         <f>MAX(D40,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="E41" s="19">
         <f>MAX(E40,$C$18)</f>
-        <v/>
+        <v>161.3963062</v>
       </c>
       <c r="F41" s="19">
         <f>MAX(F40,$C$18)</f>
-        <v/>
+        <v>188.8183213</v>
       </c>
     </row>
     <row r="42">
@@ -6552,19 +6552,19 @@
       </c>
       <c r="C42" s="19">
         <f>ROUNDUP(C41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D42" s="19">
         <f>ROUNDUP(D41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E42" s="19">
         <f>ROUNDUP(E41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F42" s="19">
         <f>ROUNDUP(F41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -6584,21 +6584,21 @@
           <t>Vu &lt;= phi 1.1 Vc ?</t>
         </is>
       </c>
-      <c r="C44" s="18">
+      <c r="C44" s="18" t="str">
         <f>IF(C28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="D44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="D44" s="18" t="str">
         <f>IF(D28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="E44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="E44" s="18" t="str">
         <f>IF(E28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="F44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="F44" s="18" t="str">
         <f>IF(F28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
+        <v>Si - sin estribos</v>
       </c>
     </row>
     <row r="45">
@@ -6607,21 +6607,21 @@
           <t>CHECK deflexion (h&gt;=Ln/18.5)</t>
         </is>
       </c>
-      <c r="C45" s="18">
+      <c r="C45" s="18" t="str">
         <f>IF($C$8&gt;=C24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="D45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="D45" s="18" t="str">
         <f>IF($C$8&gt;=D24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="E45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="E45" s="18" t="str">
         <f>IF($C$8&gt;=E24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="F45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="F45" s="18" t="str">
         <f>IF($C$8&gt;=F24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
   </sheetData>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="C16" s="19">
         <f>C8*1000-C11*1000-C12/2</f>
-        <v/>
+        <v>303.65</v>
       </c>
     </row>
     <row r="17">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="C17" s="19">
         <f>(1.2*C14+1.6*C15)*C10</f>
-        <v/>
+        <v>10.60096</v>
       </c>
     </row>
     <row r="18">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="C18" s="21">
         <f>MAX(0.25*SQRT(C5)/C6,1.4/C6)*C7*1000*C16</f>
-        <v/>
+        <v>151.825</v>
       </c>
     </row>
     <row r="19">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="C19" s="21">
         <f>0.17*SQRT(C5)*C7*1000*C16/1000</f>
-        <v/>
+        <v>40.97250167</v>
       </c>
     </row>
     <row r="20">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="C20" s="21">
         <f>0.75*1.1*C19</f>
-        <v/>
+        <v>33.80231387</v>
       </c>
     </row>
     <row r="22">
@@ -6906,19 +6906,19 @@
       </c>
       <c r="C25" s="19">
         <f>MIN(C24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>462.5</v>
       </c>
       <c r="D25" s="19">
         <f>MIN(D24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E25" s="19">
         <f>MIN(E24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="F25" s="19">
         <f>MIN(F24*1000/4,$C$7*1000+16*$C$9*1000,$C$10*1000)</f>
-        <v/>
+        <v>800</v>
       </c>
     </row>
     <row r="26">
@@ -6929,19 +6929,19 @@
       </c>
       <c r="C26" s="19">
         <f>$C$17*C24^2/10</f>
-        <v/>
+        <v>3.62817856</v>
       </c>
       <c r="D26" s="19">
         <f>$C$17*D24^2/10</f>
-        <v/>
+        <v>11.197264</v>
       </c>
       <c r="E26" s="19">
         <f>$C$17*E24^2/10</f>
-        <v/>
+        <v>20.99255104</v>
       </c>
       <c r="F26" s="19">
         <f>$C$17*F24^2/10</f>
-        <v/>
+        <v>24.42461184</v>
       </c>
     </row>
     <row r="27">
@@ -6952,19 +6952,19 @@
       </c>
       <c r="C27" s="19">
         <f>$C$17*C24^2/14</f>
-        <v/>
+        <v>2.591556114</v>
       </c>
       <c r="D27" s="19">
         <f>$C$17*D24^2/14</f>
-        <v/>
+        <v>7.998045714</v>
       </c>
       <c r="E27" s="19">
         <f>$C$17*E24^2/14</f>
-        <v/>
+        <v>14.99467931</v>
       </c>
       <c r="F27" s="19">
         <f>$C$17*F24^2/14</f>
-        <v/>
+        <v>17.44615131</v>
       </c>
     </row>
     <row r="28">
@@ -6975,19 +6975,19 @@
       </c>
       <c r="C28" s="19">
         <f>1.15*$C$17*C24/2</f>
-        <v/>
+        <v>11.2767712</v>
       </c>
       <c r="D28" s="19">
         <f>1.15*$C$17*D24/2</f>
-        <v/>
+        <v>19.810544</v>
       </c>
       <c r="E28" s="19">
         <f>1.15*$C$17*E24/2</f>
-        <v/>
+        <v>27.1252064</v>
       </c>
       <c r="F28" s="19">
         <f>1.15*$C$17*F24/2</f>
-        <v/>
+        <v>29.2586496</v>
       </c>
     </row>
     <row r="29">
@@ -7009,19 +7009,19 @@
       </c>
       <c r="C30" s="16">
         <f>C27*1000000/(0.9*C25*$C$16^2)</f>
-        <v/>
+        <v>0.06752425472</v>
       </c>
       <c r="D30" s="16">
         <f>D27*1000000/(0.9*D25*$C$16^2)</f>
-        <v/>
+        <v>0.1204771859</v>
       </c>
       <c r="E30" s="16">
         <f>E27*1000000/(0.9*E25*$C$16^2)</f>
-        <v/>
+        <v>0.2258697727</v>
       </c>
       <c r="F30" s="16">
         <f>F27*1000000/(0.9*F25*$C$16^2)</f>
-        <v/>
+        <v>0.2627970995</v>
       </c>
     </row>
     <row r="31">
@@ -7032,19 +7032,19 @@
       </c>
       <c r="C31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*C30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0001610007519</v>
       </c>
       <c r="D31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*D30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0002875801693</v>
       </c>
       <c r="E31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*E30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0005403615608</v>
       </c>
       <c r="F31" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*F30/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0006292005562</v>
       </c>
     </row>
     <row r="32">
@@ -7055,19 +7055,19 @@
       </c>
       <c r="C32" s="16">
         <f>C31*C25*$C$16</f>
-        <v/>
+        <v>22.61064372</v>
       </c>
       <c r="D32" s="16">
         <f>D31*D25*$C$16</f>
-        <v/>
+        <v>69.85897472</v>
       </c>
       <c r="E32" s="16">
         <f>E31*E25*$C$16</f>
-        <v/>
+        <v>131.2646304</v>
       </c>
       <c r="F32" s="16">
         <f>F31*F25*$C$16</f>
-        <v/>
+        <v>152.8453991</v>
       </c>
     </row>
     <row r="33">
@@ -7078,19 +7078,19 @@
       </c>
       <c r="C33" s="16">
         <f>C32*$C$6/(0.85*$C$5*C25)</f>
-        <v/>
+        <v>0.8627272644</v>
       </c>
       <c r="D33" s="16">
         <f>D32*$C$6/(0.85*$C$5*D25)</f>
-        <v/>
+        <v>1.541006795</v>
       </c>
       <c r="E33" s="16">
         <f>E32*$C$6/(0.85*$C$5*E25)</f>
-        <v/>
+        <v>2.895543317</v>
       </c>
       <c r="F33" s="16">
         <f>F32*$C$6/(0.85*$C$5*F25)</f>
-        <v/>
+        <v>3.371589686</v>
       </c>
     </row>
     <row r="34">
@@ -7099,21 +7099,21 @@
           <t>a &lt;= hf ? (viga T)</t>
         </is>
       </c>
-      <c r="C34" s="18">
+      <c r="C34" s="18" t="str">
         <f>IF(C33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="D34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="D34" s="18" t="str">
         <f>IF(D33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="E34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="E34" s="18" t="str">
         <f>IF(E33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
-      </c>
-      <c r="F34" s="18">
+        <v>Si (T)</v>
+      </c>
+      <c r="F34" s="18" t="str">
         <f>IF(F33&lt;=$C$9*1000,"Si (T)","revisar")</f>
-        <v/>
+        <v>Si (T)</v>
       </c>
     </row>
     <row r="35">
@@ -7124,19 +7124,19 @@
       </c>
       <c r="C35" s="19">
         <f>MAX(C32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="D35" s="19">
         <f>MAX(D32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="E35" s="19">
         <f>MAX(E32,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="F35" s="19">
         <f>MAX(F32,$C$18)</f>
-        <v/>
+        <v>152.8453991</v>
       </c>
     </row>
     <row r="36">
@@ -7147,19 +7147,19 @@
       </c>
       <c r="C36" s="19">
         <f>ROUNDUP(C35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D36" s="19">
         <f>ROUNDUP(D35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E36" s="19">
         <f>ROUNDUP(E35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F36" s="19">
         <f>ROUNDUP(F35/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -7181,19 +7181,19 @@
       </c>
       <c r="C38" s="16">
         <f>C26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>0.2914796996</v>
       </c>
       <c r="D38" s="16">
         <f>D26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>0.8995629881</v>
       </c>
       <c r="E38" s="16">
         <f>E26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>1.686494303</v>
       </c>
       <c r="F38" s="16">
         <f>F26*1000000/(0.9*$C$7*1000*$C$16^2)</f>
-        <v/>
+        <v>1.962218343</v>
       </c>
     </row>
     <row r="39">
@@ -7204,19 +7204,19 @@
       </c>
       <c r="C39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*C38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.0006983018625</v>
       </c>
       <c r="D39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*D38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.002183899739</v>
       </c>
       <c r="E39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*E38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.004168806263</v>
       </c>
       <c r="F39" s="16">
         <f>(0.85*$C$5/$C$6)*(1-SQRT(1-2*F38/(0.85*$C$5)))</f>
-        <v/>
+        <v>0.004882271123</v>
       </c>
     </row>
     <row r="40">
@@ -7227,19 +7227,19 @@
       </c>
       <c r="C40" s="16">
         <f>C39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>31.80590408</v>
       </c>
       <c r="D40" s="16">
         <f>D39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>99.47117335</v>
       </c>
       <c r="E40" s="16">
         <f>E39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>189.8787033</v>
       </c>
       <c r="F40" s="16">
         <f>F39*$C$7*1000*$C$16</f>
-        <v/>
+        <v>222.375244</v>
       </c>
     </row>
     <row r="41">
@@ -7250,19 +7250,19 @@
       </c>
       <c r="C41" s="19">
         <f>MAX(C40,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="D41" s="19">
         <f>MAX(D40,$C$18)</f>
-        <v/>
+        <v>151.825</v>
       </c>
       <c r="E41" s="19">
         <f>MAX(E40,$C$18)</f>
-        <v/>
+        <v>189.8787033</v>
       </c>
       <c r="F41" s="19">
         <f>MAX(F40,$C$18)</f>
-        <v/>
+        <v>222.375244</v>
       </c>
     </row>
     <row r="42">
@@ -7273,19 +7273,19 @@
       </c>
       <c r="C42" s="19">
         <f>ROUNDUP(C41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="D42" s="19">
         <f>ROUNDUP(D41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="E42" s="19">
         <f>ROUNDUP(E41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="F42" s="19">
         <f>ROUNDUP(F41/$C$13,0)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -7305,21 +7305,21 @@
           <t>Vu &lt;= phi 1.1 Vc ?</t>
         </is>
       </c>
-      <c r="C44" s="18">
+      <c r="C44" s="18" t="str">
         <f>IF(C28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="D44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="D44" s="18" t="str">
         <f>IF(D28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="E44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="E44" s="18" t="str">
         <f>IF(E28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
-      </c>
-      <c r="F44" s="18">
+        <v>Si - sin estribos</v>
+      </c>
+      <c r="F44" s="18" t="str">
         <f>IF(F28&lt;=$C$20,"Si - sin estribos","Requiere estribos")</f>
-        <v/>
+        <v>Si - sin estribos</v>
       </c>
     </row>
     <row r="45">
@@ -7328,21 +7328,21 @@
           <t>CHECK deflexion (h&gt;=Ln/18.5)</t>
         </is>
       </c>
-      <c r="C45" s="18">
+      <c r="C45" s="18" t="str">
         <f>IF($C$8&gt;=C24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="D45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="D45" s="18" t="str">
         <f>IF($C$8&gt;=D24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="E45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="E45" s="18" t="str">
         <f>IF($C$8&gt;=E24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
-      </c>
-      <c r="F45" s="18">
+        <v>CUMPLE</v>
+      </c>
+      <c r="F45" s="18" t="str">
         <f>IF($C$8&gt;=F24/18.5,"CUMPLE","REVISAR")</f>
-        <v/>
+        <v>CUMPLE</v>
       </c>
     </row>
   </sheetData>

</xml_diff>